<commit_message>
Adjustments and additions have been made to the product backlog
</commit_message>
<xml_diff>
--- a/docs/Product_Backlog.xlsx
+++ b/docs/Product_Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java项目\EBU6304-Group17\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0E093B-1ACC-48DA-A053-EFE4EDE76171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DBCD1AB-1E0A-4ECD-A8BA-721446DDE501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2716,32 +2716,32 @@
       <c r="J43" s="42"/>
     </row>
     <row r="44" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="14" t="s">
+      <c r="A44" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="B44" s="15" t="s">
+      <c r="B44" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="21" t="s">
         <v>183</v>
       </c>
       <c r="D44" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="E44" s="14">
+      <c r="E44" s="19">
         <v>4</v>
       </c>
-      <c r="F44" s="16" t="s">
+      <c r="F44" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="G44" s="14">
-        <v>2</v>
-      </c>
-      <c r="H44" s="15" t="s">
+      <c r="G44" s="19">
+        <v>2</v>
+      </c>
+      <c r="H44" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="I44" s="18"/>
-      <c r="J44" s="18"/>
+      <c r="I44" s="22"/>
+      <c r="J44" s="22"/>
     </row>
     <row r="45" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="43" t="s">
@@ -2770,30 +2770,30 @@
       <c r="J45" s="46"/>
     </row>
     <row r="46" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="14" t="s">
+      <c r="A46" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="B46" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="21" t="s">
         <v>193</v>
       </c>
       <c r="D46" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="E46" s="14">
+      <c r="E46" s="19">
         <v>4</v>
       </c>
-      <c r="F46" s="16" t="s">
+      <c r="F46" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="G46" s="14">
-        <v>1</v>
-      </c>
-      <c r="H46" s="15"/>
-      <c r="I46" s="18"/>
-      <c r="J46" s="18"/>
+      <c r="G46" s="19">
+        <v>1</v>
+      </c>
+      <c r="H46" s="20"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22"/>
     </row>
     <row r="47" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="43" t="s">
@@ -2822,30 +2822,30 @@
       <c r="J47" s="46"/>
     </row>
     <row r="48" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="14" t="s">
+      <c r="A48" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B48" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="C48" s="21" t="s">
         <v>201</v>
       </c>
       <c r="D48" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="E48" s="14">
+      <c r="E48" s="19">
         <v>4</v>
       </c>
-      <c r="F48" s="16" t="s">
+      <c r="F48" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G48" s="14">
-        <v>1</v>
-      </c>
-      <c r="H48" s="15"/>
-      <c r="I48" s="18"/>
-      <c r="J48" s="18"/>
+      <c r="G48" s="19">
+        <v>1</v>
+      </c>
+      <c r="H48" s="20"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
     </row>
     <row r="49" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="43" t="s">
@@ -2874,30 +2874,30 @@
       <c r="J49" s="46"/>
     </row>
     <row r="50" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="14" t="s">
+      <c r="A50" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B50" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="21" t="s">
         <v>209</v>
       </c>
       <c r="D50" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="E50" s="14">
+      <c r="E50" s="19">
         <v>4</v>
       </c>
-      <c r="F50" s="16" t="s">
+      <c r="F50" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="G50" s="14">
-        <v>2</v>
-      </c>
-      <c r="H50" s="15"/>
-      <c r="I50" s="18"/>
-      <c r="J50" s="18"/>
+      <c r="G50" s="19">
+        <v>2</v>
+      </c>
+      <c r="H50" s="20"/>
+      <c r="I50" s="22"/>
+      <c r="J50" s="22"/>
     </row>
     <row r="51" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="43" t="s">

</xml_diff>